<commit_message>
References: Kemeny (1959) confirmed on JSTOR; no entry left to verify
The author read JSTOR 20026529 in a browser: the article starts on page
577 and runs 15 pages, so 577-591, as in the entry. The 571 given by some
citing papers is wrong. The last verify flag is removed: all 98 entries
are now confirmed by their official record.

The printed bibliography does not change, so the PDF of record stays as
it is; the concept map is regenerated (its "Still to verify" column).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B9JazvqpAeMRrMi1Y9nCDd
</commit_message>
<xml_diff>
--- a/literature/concept-map/concept-map.xlsx
+++ b/literature/concept-map/concept-map.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1328" uniqueCount="892">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="891">
   <si>
     <t xml:space="preserve">Concept map of the note “Voting for a consensus with veto rights” (v0.1)</t>
   </si>
@@ -1830,9 +1830,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.jstor.org/stable/20026529</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not checked against the journal's record: no Crossref record, and JSTOR 20026529 refuses automated access. First page 577 in Fishburn (1977), the earliest citing paper found, and in Kondratev and Nesterov (2020); 571 in Young and Levenglick (1978), Young (1988) and Bartholdi et al. (1989)</t>
   </si>
   <si>
     <t xml:space="preserve">Kondratev &amp; Ianovski (2024). Veto Core Consistent Preference Aggregation</t>
@@ -5900,7 +5897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
         <v>542</v>
       </c>
@@ -5922,9 +5919,7 @@
       <c r="G57" s="9" t="s">
         <v>546</v>
       </c>
-      <c r="H57" s="8" t="s">
-        <v>547</v>
-      </c>
+      <c r="H57" s="8"/>
       <c r="I57" s="8" t="n">
         <f aca="false">COUNTIF(INDEX(Matrix!$C$3:$AK$100,MATCH(D57,Matrix!$B$3:$B$100,0),0),"x")</f>
         <v>1</v>
@@ -5932,25 +5927,25 @@
     </row>
     <row r="58" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
+        <v>547</v>
+      </c>
+      <c r="B58" s="8" t="s">
         <v>548</v>
       </c>
-      <c r="B58" s="8" t="s">
+      <c r="C58" s="8" t="s">
         <v>549</v>
       </c>
-      <c r="C58" s="8" t="s">
+      <c r="D58" s="8" t="s">
         <v>550</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>551</v>
       </c>
       <c r="E58" s="8" t="s">
         <v>206</v>
       </c>
       <c r="F58" s="8" t="s">
+        <v>551</v>
+      </c>
+      <c r="G58" s="9" t="s">
         <v>552</v>
-      </c>
-      <c r="G58" s="9" t="s">
-        <v>553</v>
       </c>
       <c r="H58" s="8"/>
       <c r="I58" s="8" t="n">
@@ -5963,22 +5958,22 @@
         <v>151</v>
       </c>
       <c r="B59" s="8" t="s">
+        <v>553</v>
+      </c>
+      <c r="C59" s="8" t="s">
         <v>554</v>
       </c>
-      <c r="C59" s="8" t="s">
+      <c r="D59" s="8" t="s">
         <v>555</v>
-      </c>
-      <c r="D59" s="8" t="s">
-        <v>556</v>
       </c>
       <c r="E59" s="8" t="s">
         <v>237</v>
       </c>
       <c r="F59" s="8" t="s">
+        <v>556</v>
+      </c>
+      <c r="G59" s="9" t="s">
         <v>557</v>
-      </c>
-      <c r="G59" s="9" t="s">
-        <v>558</v>
       </c>
       <c r="H59" s="8"/>
       <c r="I59" s="8" t="n">
@@ -5988,25 +5983,25 @@
     </row>
     <row r="60" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="B60" s="8" t="s">
         <v>559</v>
       </c>
-      <c r="B60" s="8" t="s">
+      <c r="C60" s="8" t="s">
         <v>560</v>
       </c>
-      <c r="C60" s="8" t="s">
+      <c r="D60" s="8" t="s">
         <v>561</v>
-      </c>
-      <c r="D60" s="8" t="s">
-        <v>562</v>
       </c>
       <c r="E60" s="8" t="s">
         <v>349</v>
       </c>
       <c r="F60" s="8" t="s">
+        <v>562</v>
+      </c>
+      <c r="G60" s="9" t="s">
         <v>563</v>
-      </c>
-      <c r="G60" s="9" t="s">
-        <v>564</v>
       </c>
       <c r="H60" s="8"/>
       <c r="I60" s="8" t="n">
@@ -6016,25 +6011,25 @@
     </row>
     <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
+        <v>564</v>
+      </c>
+      <c r="B61" s="8" t="s">
         <v>565</v>
       </c>
-      <c r="B61" s="8" t="s">
+      <c r="C61" s="8" t="s">
         <v>566</v>
       </c>
-      <c r="C61" s="8" t="s">
+      <c r="D61" s="8" t="s">
         <v>567</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>568</v>
       </c>
       <c r="E61" s="8" t="s">
         <v>281</v>
       </c>
       <c r="F61" s="8" t="s">
+        <v>568</v>
+      </c>
+      <c r="G61" s="9" t="s">
         <v>569</v>
-      </c>
-      <c r="G61" s="9" t="s">
-        <v>570</v>
       </c>
       <c r="H61" s="8"/>
       <c r="I61" s="8" t="n">
@@ -6044,25 +6039,25 @@
     </row>
     <row r="62" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B62" s="8" t="s">
         <v>203</v>
       </c>
       <c r="C62" s="8" t="s">
+        <v>571</v>
+      </c>
+      <c r="D62" s="8" t="s">
         <v>572</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>573</v>
       </c>
       <c r="E62" s="8" t="s">
         <v>206</v>
       </c>
       <c r="F62" s="8" t="s">
+        <v>573</v>
+      </c>
+      <c r="G62" s="9" t="s">
         <v>574</v>
-      </c>
-      <c r="G62" s="9" t="s">
-        <v>575</v>
       </c>
       <c r="H62" s="8"/>
       <c r="I62" s="8" t="n">
@@ -6072,25 +6067,25 @@
     </row>
     <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B63" s="8" t="s">
         <v>241</v>
       </c>
       <c r="C63" s="8" t="s">
+        <v>576</v>
+      </c>
+      <c r="D63" s="8" t="s">
         <v>577</v>
-      </c>
-      <c r="D63" s="8" t="s">
-        <v>578</v>
       </c>
       <c r="E63" s="8" t="s">
         <v>281</v>
       </c>
       <c r="F63" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="G63" s="9" t="s">
         <v>579</v>
-      </c>
-      <c r="G63" s="9" t="s">
-        <v>580</v>
       </c>
       <c r="H63" s="8"/>
       <c r="I63" s="8" t="n">
@@ -6100,25 +6095,25 @@
     </row>
     <row r="64" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
+        <v>580</v>
+      </c>
+      <c r="B64" s="8" t="s">
         <v>581</v>
       </c>
-      <c r="B64" s="8" t="s">
+      <c r="C64" s="8" t="s">
         <v>582</v>
       </c>
-      <c r="C64" s="8" t="s">
+      <c r="D64" s="8" t="s">
         <v>583</v>
-      </c>
-      <c r="D64" s="8" t="s">
-        <v>584</v>
       </c>
       <c r="E64" s="8" t="s">
         <v>281</v>
       </c>
       <c r="F64" s="8" t="s">
+        <v>584</v>
+      </c>
+      <c r="G64" s="9" t="s">
         <v>585</v>
-      </c>
-      <c r="G64" s="9" t="s">
-        <v>586</v>
       </c>
       <c r="H64" s="8"/>
       <c r="I64" s="8" t="n">
@@ -6128,25 +6123,25 @@
     </row>
     <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B65" s="8" t="s">
         <v>253</v>
       </c>
       <c r="C65" s="8" t="s">
+        <v>587</v>
+      </c>
+      <c r="D65" s="8" t="s">
         <v>588</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>589</v>
       </c>
       <c r="E65" s="8" t="s">
         <v>206</v>
       </c>
       <c r="F65" s="8" t="s">
+        <v>589</v>
+      </c>
+      <c r="G65" s="9" t="s">
         <v>590</v>
-      </c>
-      <c r="G65" s="9" t="s">
-        <v>591</v>
       </c>
       <c r="H65" s="8"/>
       <c r="I65" s="8" t="n">
@@ -6156,25 +6151,25 @@
     </row>
     <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="B66" s="8" t="s">
         <v>592</v>
       </c>
-      <c r="B66" s="8" t="s">
+      <c r="C66" s="8" t="s">
         <v>593</v>
       </c>
-      <c r="C66" s="8" t="s">
+      <c r="D66" s="8" t="s">
         <v>594</v>
       </c>
-      <c r="D66" s="8" t="s">
+      <c r="E66" s="8" t="s">
         <v>595</v>
       </c>
-      <c r="E66" s="8" t="s">
+      <c r="F66" s="8" t="s">
         <v>596</v>
       </c>
-      <c r="F66" s="8" t="s">
+      <c r="G66" s="9" t="s">
         <v>597</v>
-      </c>
-      <c r="G66" s="9" t="s">
-        <v>598</v>
       </c>
       <c r="H66" s="8"/>
       <c r="I66" s="8" t="n">
@@ -6184,25 +6179,25 @@
     </row>
     <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>592</v>
+      </c>
+      <c r="C67" s="8" t="s">
         <v>599</v>
       </c>
-      <c r="B67" s="8" t="s">
-        <v>593</v>
-      </c>
-      <c r="C67" s="8" t="s">
+      <c r="D67" s="8" t="s">
         <v>600</v>
       </c>
-      <c r="D67" s="8" t="s">
+      <c r="E67" s="8" t="s">
         <v>601</v>
       </c>
-      <c r="E67" s="8" t="s">
+      <c r="F67" s="8" t="s">
         <v>602</v>
       </c>
-      <c r="F67" s="8" t="s">
+      <c r="G67" s="9" t="s">
         <v>603</v>
-      </c>
-      <c r="G67" s="9" t="s">
-        <v>604</v>
       </c>
       <c r="H67" s="8"/>
       <c r="I67" s="8" t="n">
@@ -6212,25 +6207,25 @@
     </row>
     <row r="68" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
+        <v>604</v>
+      </c>
+      <c r="B68" s="8" t="s">
         <v>605</v>
       </c>
-      <c r="B68" s="8" t="s">
+      <c r="C68" s="8" t="s">
         <v>606</v>
       </c>
-      <c r="C68" s="8" t="s">
+      <c r="D68" s="8" t="s">
         <v>607</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>608</v>
       </c>
       <c r="E68" s="8" t="s">
         <v>237</v>
       </c>
       <c r="F68" s="8" t="s">
+        <v>608</v>
+      </c>
+      <c r="G68" s="9" t="s">
         <v>609</v>
-      </c>
-      <c r="G68" s="9" t="s">
-        <v>610</v>
       </c>
       <c r="H68" s="8"/>
       <c r="I68" s="8" t="n">
@@ -6240,25 +6235,25 @@
     </row>
     <row r="69" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
+        <v>610</v>
+      </c>
+      <c r="B69" s="8" t="s">
         <v>611</v>
       </c>
-      <c r="B69" s="8" t="s">
+      <c r="C69" s="8" t="s">
         <v>612</v>
       </c>
-      <c r="C69" s="8" t="s">
+      <c r="D69" s="8" t="s">
         <v>613</v>
       </c>
-      <c r="D69" s="8" t="s">
+      <c r="E69" s="8" t="s">
         <v>614</v>
       </c>
-      <c r="E69" s="8" t="s">
+      <c r="F69" s="8" t="s">
         <v>615</v>
       </c>
-      <c r="F69" s="8" t="s">
+      <c r="G69" s="9" t="s">
         <v>616</v>
-      </c>
-      <c r="G69" s="9" t="s">
-        <v>617</v>
       </c>
       <c r="H69" s="8"/>
       <c r="I69" s="8" t="n">
@@ -6268,25 +6263,25 @@
     </row>
     <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
+        <v>617</v>
+      </c>
+      <c r="B70" s="8" t="s">
         <v>618</v>
       </c>
-      <c r="B70" s="8" t="s">
+      <c r="C70" s="8" t="s">
         <v>619</v>
       </c>
-      <c r="C70" s="8" t="s">
+      <c r="D70" s="8" t="s">
         <v>620</v>
       </c>
-      <c r="D70" s="8" t="s">
+      <c r="E70" s="8" t="s">
         <v>621</v>
       </c>
-      <c r="E70" s="8" t="s">
+      <c r="F70" s="8" t="s">
         <v>622</v>
       </c>
-      <c r="F70" s="8" t="s">
+      <c r="G70" s="9" t="s">
         <v>623</v>
-      </c>
-      <c r="G70" s="9" t="s">
-        <v>624</v>
       </c>
       <c r="H70" s="8"/>
       <c r="I70" s="8" t="n">
@@ -6296,25 +6291,25 @@
     </row>
     <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B71" s="8" t="s">
         <v>310</v>
       </c>
       <c r="C71" s="8" t="s">
+        <v>625</v>
+      </c>
+      <c r="D71" s="8" t="s">
         <v>626</v>
       </c>
-      <c r="D71" s="8" t="s">
+      <c r="E71" s="8" t="s">
         <v>627</v>
       </c>
-      <c r="E71" s="8" t="s">
+      <c r="F71" s="8" t="s">
         <v>628</v>
       </c>
-      <c r="F71" s="8" t="s">
+      <c r="G71" s="9" t="s">
         <v>629</v>
-      </c>
-      <c r="G71" s="9" t="s">
-        <v>630</v>
       </c>
       <c r="H71" s="8"/>
       <c r="I71" s="8" t="n">
@@ -6324,25 +6319,25 @@
     </row>
     <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B72" s="8" t="s">
         <v>525</v>
       </c>
       <c r="C72" s="8" t="s">
+        <v>631</v>
+      </c>
+      <c r="D72" s="8" t="s">
         <v>632</v>
       </c>
-      <c r="D72" s="8" t="s">
+      <c r="E72" s="8" t="s">
         <v>633</v>
       </c>
-      <c r="E72" s="8" t="s">
+      <c r="F72" s="8" t="s">
         <v>634</v>
       </c>
-      <c r="F72" s="8" t="s">
+      <c r="G72" s="9" t="s">
         <v>635</v>
-      </c>
-      <c r="G72" s="9" t="s">
-        <v>636</v>
       </c>
       <c r="H72" s="8"/>
       <c r="I72" s="8" t="n">
@@ -6352,25 +6347,25 @@
     </row>
     <row r="73" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="B73" s="8" t="s">
         <v>637</v>
       </c>
-      <c r="B73" s="8" t="s">
+      <c r="C73" s="8" t="s">
         <v>638</v>
       </c>
-      <c r="C73" s="8" t="s">
+      <c r="D73" s="8" t="s">
         <v>639</v>
       </c>
-      <c r="D73" s="8" t="s">
+      <c r="E73" s="8" t="s">
+        <v>633</v>
+      </c>
+      <c r="F73" s="8" t="s">
         <v>640</v>
       </c>
-      <c r="E73" s="8" t="s">
-        <v>634</v>
-      </c>
-      <c r="F73" s="8" t="s">
+      <c r="G73" s="9" t="s">
         <v>641</v>
-      </c>
-      <c r="G73" s="9" t="s">
-        <v>642</v>
       </c>
       <c r="H73" s="8"/>
       <c r="I73" s="8" t="n">
@@ -6380,22 +6375,22 @@
     </row>
     <row r="74" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="B74" s="8" t="s">
         <v>643</v>
       </c>
-      <c r="B74" s="8" t="s">
+      <c r="C74" s="8" t="s">
         <v>644</v>
       </c>
-      <c r="C74" s="8" t="s">
+      <c r="D74" s="8" t="s">
         <v>645</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>646</v>
       </c>
       <c r="E74" s="8" t="s">
         <v>206</v>
       </c>
       <c r="F74" s="8" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="G74" s="8"/>
       <c r="H74" s="8"/>
@@ -6406,25 +6401,25 @@
     </row>
     <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="B75" s="8" t="s">
         <v>648</v>
       </c>
-      <c r="B75" s="8" t="s">
+      <c r="C75" s="8" t="s">
         <v>649</v>
       </c>
-      <c r="C75" s="8" t="s">
+      <c r="D75" s="8" t="s">
         <v>650</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>651</v>
       </c>
       <c r="E75" s="8" t="s">
         <v>237</v>
       </c>
       <c r="F75" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="G75" s="9" t="s">
         <v>652</v>
-      </c>
-      <c r="G75" s="9" t="s">
-        <v>653</v>
       </c>
       <c r="H75" s="8"/>
       <c r="I75" s="8" t="n">
@@ -6434,25 +6429,25 @@
     </row>
     <row r="76" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
+        <v>653</v>
+      </c>
+      <c r="B76" s="8" t="s">
         <v>654</v>
       </c>
-      <c r="B76" s="8" t="s">
+      <c r="C76" s="8" t="s">
         <v>655</v>
       </c>
-      <c r="C76" s="8" t="s">
+      <c r="D76" s="8" t="s">
         <v>656</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>657</v>
       </c>
       <c r="E76" s="8" t="s">
         <v>206</v>
       </c>
       <c r="F76" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="G76" s="9" t="s">
         <v>658</v>
-      </c>
-      <c r="G76" s="9" t="s">
-        <v>659</v>
       </c>
       <c r="H76" s="8"/>
       <c r="I76" s="8" t="n">
@@ -6462,25 +6457,25 @@
     </row>
     <row r="77" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="B77" s="8" t="s">
         <v>660</v>
       </c>
-      <c r="B77" s="8" t="s">
+      <c r="C77" s="8" t="s">
         <v>661</v>
       </c>
-      <c r="C77" s="8" t="s">
+      <c r="D77" s="8" t="s">
         <v>662</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>663</v>
       </c>
       <c r="E77" s="8" t="s">
         <v>237</v>
       </c>
       <c r="F77" s="8" t="s">
+        <v>663</v>
+      </c>
+      <c r="G77" s="9" t="s">
         <v>664</v>
-      </c>
-      <c r="G77" s="9" t="s">
-        <v>665</v>
       </c>
       <c r="H77" s="8"/>
       <c r="I77" s="8" t="n">
@@ -6490,25 +6485,25 @@
     </row>
     <row r="78" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
+        <v>665</v>
+      </c>
+      <c r="B78" s="8" t="s">
         <v>666</v>
       </c>
-      <c r="B78" s="8" t="s">
+      <c r="C78" s="8" t="s">
         <v>667</v>
       </c>
-      <c r="C78" s="8" t="s">
+      <c r="D78" s="8" t="s">
         <v>668</v>
       </c>
-      <c r="D78" s="8" t="s">
+      <c r="E78" s="8" t="s">
         <v>669</v>
       </c>
-      <c r="E78" s="8" t="s">
+      <c r="F78" s="8" t="s">
         <v>670</v>
       </c>
-      <c r="F78" s="8" t="s">
+      <c r="G78" s="9" t="s">
         <v>671</v>
-      </c>
-      <c r="G78" s="9" t="s">
-        <v>672</v>
       </c>
       <c r="H78" s="8"/>
       <c r="I78" s="8" t="n">
@@ -6518,25 +6513,25 @@
     </row>
     <row r="79" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B79" s="8" t="s">
         <v>304</v>
       </c>
       <c r="C79" s="8" t="s">
+        <v>673</v>
+      </c>
+      <c r="D79" s="8" t="s">
         <v>674</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>675</v>
       </c>
       <c r="E79" s="8" t="s">
         <v>206</v>
       </c>
       <c r="F79" s="8" t="s">
+        <v>675</v>
+      </c>
+      <c r="G79" s="9" t="s">
         <v>676</v>
-      </c>
-      <c r="G79" s="9" t="s">
-        <v>677</v>
       </c>
       <c r="H79" s="8"/>
       <c r="I79" s="8" t="n">
@@ -6546,25 +6541,25 @@
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
+        <v>677</v>
+      </c>
+      <c r="B80" s="8" t="s">
         <v>678</v>
       </c>
-      <c r="B80" s="8" t="s">
+      <c r="C80" s="8" t="s">
         <v>679</v>
       </c>
-      <c r="C80" s="8" t="s">
+      <c r="D80" s="8" t="s">
         <v>680</v>
-      </c>
-      <c r="D80" s="8" t="s">
-        <v>681</v>
       </c>
       <c r="E80" s="8" t="s">
         <v>237</v>
       </c>
       <c r="F80" s="8" t="s">
+        <v>681</v>
+      </c>
+      <c r="G80" s="9" t="s">
         <v>682</v>
-      </c>
-      <c r="G80" s="9" t="s">
-        <v>683</v>
       </c>
       <c r="H80" s="8"/>
       <c r="I80" s="8" t="n">
@@ -6574,25 +6569,25 @@
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
+        <v>683</v>
+      </c>
+      <c r="B81" s="8" t="s">
         <v>684</v>
       </c>
-      <c r="B81" s="8" t="s">
+      <c r="C81" s="8" t="s">
         <v>685</v>
       </c>
-      <c r="C81" s="8" t="s">
+      <c r="D81" s="8" t="s">
         <v>686</v>
-      </c>
-      <c r="D81" s="8" t="s">
-        <v>687</v>
       </c>
       <c r="E81" s="8" t="s">
         <v>237</v>
       </c>
       <c r="F81" s="8" t="s">
+        <v>687</v>
+      </c>
+      <c r="G81" s="9" t="s">
         <v>688</v>
-      </c>
-      <c r="G81" s="9" t="s">
-        <v>689</v>
       </c>
       <c r="H81" s="8"/>
       <c r="I81" s="8" t="n">
@@ -6602,25 +6597,25 @@
     </row>
     <row r="82" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B82" s="8" t="s">
         <v>441</v>
       </c>
       <c r="C82" s="8" t="s">
+        <v>690</v>
+      </c>
+      <c r="D82" s="8" t="s">
         <v>691</v>
       </c>
-      <c r="D82" s="8" t="s">
+      <c r="E82" s="8" t="s">
+        <v>614</v>
+      </c>
+      <c r="F82" s="8" t="s">
         <v>692</v>
       </c>
-      <c r="E82" s="8" t="s">
-        <v>615</v>
-      </c>
-      <c r="F82" s="8" t="s">
+      <c r="G82" s="9" t="s">
         <v>693</v>
-      </c>
-      <c r="G82" s="9" t="s">
-        <v>694</v>
       </c>
       <c r="H82" s="8"/>
       <c r="I82" s="8" t="n">
@@ -6630,25 +6625,25 @@
     </row>
     <row r="83" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
+        <v>694</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>559</v>
+      </c>
+      <c r="C83" s="8" t="s">
         <v>695</v>
       </c>
-      <c r="B83" s="8" t="s">
-        <v>560</v>
-      </c>
-      <c r="C83" s="8" t="s">
+      <c r="D83" s="8" t="s">
         <v>696</v>
-      </c>
-      <c r="D83" s="8" t="s">
-        <v>697</v>
       </c>
       <c r="E83" s="8" t="s">
         <v>349</v>
       </c>
       <c r="F83" s="8" t="s">
+        <v>697</v>
+      </c>
+      <c r="G83" s="9" t="s">
         <v>698</v>
-      </c>
-      <c r="G83" s="9" t="s">
-        <v>699</v>
       </c>
       <c r="H83" s="8"/>
       <c r="I83" s="8" t="n">
@@ -6658,25 +6653,25 @@
     </row>
     <row r="84" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="B84" s="8" t="s">
         <v>700</v>
       </c>
-      <c r="B84" s="8" t="s">
+      <c r="C84" s="8" t="s">
         <v>701</v>
       </c>
-      <c r="C84" s="8" t="s">
+      <c r="D84" s="8" t="s">
         <v>702</v>
       </c>
-      <c r="D84" s="8" t="s">
+      <c r="E84" s="8" t="s">
+        <v>627</v>
+      </c>
+      <c r="F84" s="8" t="s">
         <v>703</v>
       </c>
-      <c r="E84" s="8" t="s">
-        <v>628</v>
-      </c>
-      <c r="F84" s="8" t="s">
+      <c r="G84" s="9" t="s">
         <v>704</v>
-      </c>
-      <c r="G84" s="9" t="s">
-        <v>705</v>
       </c>
       <c r="H84" s="8"/>
       <c r="I84" s="8" t="n">
@@ -6686,25 +6681,25 @@
     </row>
     <row r="85" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
+        <v>705</v>
+      </c>
+      <c r="B85" s="8" t="s">
         <v>706</v>
       </c>
-      <c r="B85" s="8" t="s">
+      <c r="C85" s="8" t="s">
         <v>707</v>
       </c>
-      <c r="C85" s="8" t="s">
+      <c r="D85" s="8" t="s">
         <v>708</v>
-      </c>
-      <c r="D85" s="8" t="s">
-        <v>709</v>
       </c>
       <c r="E85" s="8" t="s">
         <v>206</v>
       </c>
       <c r="F85" s="8" t="s">
+        <v>709</v>
+      </c>
+      <c r="G85" s="9" t="s">
         <v>710</v>
-      </c>
-      <c r="G85" s="9" t="s">
-        <v>711</v>
       </c>
       <c r="H85" s="8"/>
       <c r="I85" s="8" t="n">
@@ -6714,25 +6709,25 @@
     </row>
     <row r="86" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B86" s="8" t="s">
         <v>469</v>
       </c>
       <c r="C86" s="8" t="s">
+        <v>712</v>
+      </c>
+      <c r="D86" s="8" t="s">
         <v>713</v>
-      </c>
-      <c r="D86" s="8" t="s">
-        <v>714</v>
       </c>
       <c r="E86" s="8" t="s">
         <v>472</v>
       </c>
       <c r="F86" s="8" t="s">
+        <v>714</v>
+      </c>
+      <c r="G86" s="9" t="s">
         <v>715</v>
-      </c>
-      <c r="G86" s="9" t="s">
-        <v>716</v>
       </c>
       <c r="H86" s="8"/>
       <c r="I86" s="8" t="n">
@@ -6742,25 +6737,25 @@
     </row>
     <row r="87" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
+        <v>716</v>
+      </c>
+      <c r="B87" s="8" t="s">
         <v>717</v>
       </c>
-      <c r="B87" s="8" t="s">
+      <c r="C87" s="8" t="s">
         <v>718</v>
       </c>
-      <c r="C87" s="8" t="s">
+      <c r="D87" s="8" t="s">
         <v>719</v>
       </c>
-      <c r="D87" s="8" t="s">
+      <c r="E87" s="8" t="s">
         <v>720</v>
       </c>
-      <c r="E87" s="8" t="s">
+      <c r="F87" s="8" t="s">
         <v>721</v>
       </c>
-      <c r="F87" s="8" t="s">
+      <c r="G87" s="9" t="s">
         <v>722</v>
-      </c>
-      <c r="G87" s="9" t="s">
-        <v>723</v>
       </c>
       <c r="H87" s="8"/>
       <c r="I87" s="8" t="n">
@@ -6770,25 +6765,25 @@
     </row>
     <row r="88" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B88" s="8" t="s">
         <v>322</v>
       </c>
       <c r="C88" s="8" t="s">
+        <v>724</v>
+      </c>
+      <c r="D88" s="8" t="s">
         <v>725</v>
-      </c>
-      <c r="D88" s="8" t="s">
-        <v>726</v>
       </c>
       <c r="E88" s="8" t="s">
         <v>408</v>
       </c>
       <c r="F88" s="8" t="s">
+        <v>726</v>
+      </c>
+      <c r="G88" s="9" t="s">
         <v>727</v>
-      </c>
-      <c r="G88" s="9" t="s">
-        <v>728</v>
       </c>
       <c r="H88" s="8"/>
       <c r="I88" s="8" t="n">
@@ -6798,25 +6793,25 @@
     </row>
     <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
+        <v>728</v>
+      </c>
+      <c r="B89" s="8" t="s">
         <v>729</v>
       </c>
-      <c r="B89" s="8" t="s">
+      <c r="C89" s="8" t="s">
         <v>730</v>
       </c>
-      <c r="C89" s="8" t="s">
+      <c r="D89" s="8" t="s">
         <v>731</v>
-      </c>
-      <c r="D89" s="8" t="s">
-        <v>732</v>
       </c>
       <c r="E89" s="8" t="s">
         <v>281</v>
       </c>
       <c r="F89" s="8" t="s">
+        <v>732</v>
+      </c>
+      <c r="G89" s="9" t="s">
         <v>733</v>
-      </c>
-      <c r="G89" s="9" t="s">
-        <v>734</v>
       </c>
       <c r="H89" s="8"/>
       <c r="I89" s="8" t="n">
@@ -6826,25 +6821,25 @@
     </row>
     <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
+        <v>734</v>
+      </c>
+      <c r="B90" s="8" t="s">
         <v>735</v>
       </c>
-      <c r="B90" s="8" t="s">
+      <c r="C90" s="8" t="s">
         <v>736</v>
       </c>
-      <c r="C90" s="8" t="s">
+      <c r="D90" s="8" t="s">
         <v>737</v>
-      </c>
-      <c r="D90" s="8" t="s">
-        <v>738</v>
       </c>
       <c r="E90" s="8" t="s">
         <v>432</v>
       </c>
       <c r="F90" s="8" t="s">
+        <v>738</v>
+      </c>
+      <c r="G90" s="9" t="s">
         <v>739</v>
-      </c>
-      <c r="G90" s="9" t="s">
-        <v>740</v>
       </c>
       <c r="H90" s="8"/>
       <c r="I90" s="8" t="n">
@@ -6854,25 +6849,25 @@
     </row>
     <row r="91" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="s">
+        <v>740</v>
+      </c>
+      <c r="B91" s="8" t="s">
         <v>741</v>
       </c>
-      <c r="B91" s="8" t="s">
+      <c r="C91" s="8" t="s">
         <v>742</v>
       </c>
-      <c r="C91" s="8" t="s">
+      <c r="D91" s="8" t="s">
         <v>743</v>
       </c>
-      <c r="D91" s="8" t="s">
+      <c r="E91" s="8" t="s">
+        <v>614</v>
+      </c>
+      <c r="F91" s="8" t="s">
         <v>744</v>
       </c>
-      <c r="E91" s="8" t="s">
-        <v>615</v>
-      </c>
-      <c r="F91" s="8" t="s">
+      <c r="G91" s="9" t="s">
         <v>745</v>
-      </c>
-      <c r="G91" s="9" t="s">
-        <v>746</v>
       </c>
       <c r="H91" s="8"/>
       <c r="I91" s="8" t="n">
@@ -6882,25 +6877,25 @@
     </row>
     <row r="92" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="s">
+        <v>746</v>
+      </c>
+      <c r="B92" s="8" t="s">
         <v>747</v>
       </c>
-      <c r="B92" s="8" t="s">
+      <c r="C92" s="8" t="s">
         <v>748</v>
       </c>
-      <c r="C92" s="8" t="s">
+      <c r="D92" s="8" t="s">
         <v>749</v>
       </c>
-      <c r="D92" s="8" t="s">
+      <c r="E92" s="8" t="s">
         <v>750</v>
       </c>
-      <c r="E92" s="8" t="s">
+      <c r="F92" s="8" t="s">
         <v>751</v>
       </c>
-      <c r="F92" s="8" t="s">
+      <c r="G92" s="9" t="s">
         <v>752</v>
-      </c>
-      <c r="G92" s="9" t="s">
-        <v>753</v>
       </c>
       <c r="H92" s="8"/>
       <c r="I92" s="8" t="n">
@@ -6910,25 +6905,25 @@
     </row>
     <row r="93" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="s">
+        <v>753</v>
+      </c>
+      <c r="B93" s="8" t="s">
         <v>754</v>
       </c>
-      <c r="B93" s="8" t="s">
+      <c r="C93" s="8" t="s">
         <v>755</v>
       </c>
-      <c r="C93" s="8" t="s">
+      <c r="D93" s="8" t="s">
         <v>756</v>
-      </c>
-      <c r="D93" s="8" t="s">
-        <v>757</v>
       </c>
       <c r="E93" s="8" t="s">
         <v>237</v>
       </c>
       <c r="F93" s="8" t="s">
+        <v>757</v>
+      </c>
+      <c r="G93" s="9" t="s">
         <v>758</v>
-      </c>
-      <c r="G93" s="9" t="s">
-        <v>759</v>
       </c>
       <c r="H93" s="8"/>
       <c r="I93" s="8" t="n">
@@ -6938,25 +6933,25 @@
     </row>
     <row r="94" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="s">
+        <v>759</v>
+      </c>
+      <c r="B94" s="8" t="s">
         <v>760</v>
       </c>
-      <c r="B94" s="8" t="s">
+      <c r="C94" s="8" t="s">
         <v>761</v>
       </c>
-      <c r="C94" s="8" t="s">
+      <c r="D94" s="8" t="s">
         <v>762</v>
-      </c>
-      <c r="D94" s="8" t="s">
-        <v>763</v>
       </c>
       <c r="E94" s="8" t="s">
         <v>206</v>
       </c>
       <c r="F94" s="8" t="s">
+        <v>763</v>
+      </c>
+      <c r="G94" s="9" t="s">
         <v>764</v>
-      </c>
-      <c r="G94" s="9" t="s">
-        <v>765</v>
       </c>
       <c r="H94" s="8"/>
       <c r="I94" s="8" t="n">
@@ -6966,25 +6961,25 @@
     </row>
     <row r="95" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="B95" s="8" t="s">
+        <v>760</v>
+      </c>
+      <c r="C95" s="8" t="s">
         <v>766</v>
       </c>
-      <c r="B95" s="8" t="s">
-        <v>761</v>
-      </c>
-      <c r="C95" s="8" t="s">
+      <c r="D95" s="8" t="s">
         <v>767</v>
       </c>
-      <c r="D95" s="8" t="s">
+      <c r="E95" s="8" t="s">
         <v>768</v>
       </c>
-      <c r="E95" s="8" t="s">
+      <c r="F95" s="8" t="s">
         <v>769</v>
       </c>
-      <c r="F95" s="8" t="s">
+      <c r="G95" s="9" t="s">
         <v>770</v>
-      </c>
-      <c r="G95" s="9" t="s">
-        <v>771</v>
       </c>
       <c r="H95" s="8"/>
       <c r="I95" s="8" t="n">
@@ -6994,25 +6989,25 @@
     </row>
     <row r="96" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="7" t="s">
+        <v>771</v>
+      </c>
+      <c r="B96" s="8" t="s">
         <v>772</v>
       </c>
-      <c r="B96" s="8" t="s">
+      <c r="C96" s="8" t="s">
         <v>773</v>
       </c>
-      <c r="C96" s="8" t="s">
+      <c r="D96" s="8" t="s">
         <v>774</v>
-      </c>
-      <c r="D96" s="8" t="s">
-        <v>775</v>
       </c>
       <c r="E96" s="8" t="s">
         <v>281</v>
       </c>
       <c r="F96" s="8" t="s">
+        <v>775</v>
+      </c>
+      <c r="G96" s="9" t="s">
         <v>776</v>
-      </c>
-      <c r="G96" s="9" t="s">
-        <v>777</v>
       </c>
       <c r="H96" s="8"/>
       <c r="I96" s="8" t="n">
@@ -7022,25 +7017,25 @@
     </row>
     <row r="97" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="s">
+        <v>777</v>
+      </c>
+      <c r="B97" s="8" t="s">
         <v>778</v>
       </c>
-      <c r="B97" s="8" t="s">
+      <c r="C97" s="8" t="s">
         <v>779</v>
       </c>
-      <c r="C97" s="8" t="s">
+      <c r="D97" s="8" t="s">
         <v>780</v>
-      </c>
-      <c r="D97" s="8" t="s">
-        <v>781</v>
       </c>
       <c r="E97" s="8" t="s">
         <v>244</v>
       </c>
       <c r="F97" s="8" t="s">
+        <v>781</v>
+      </c>
+      <c r="G97" s="9" t="s">
         <v>782</v>
-      </c>
-      <c r="G97" s="9" t="s">
-        <v>783</v>
       </c>
       <c r="H97" s="8"/>
       <c r="I97" s="8" t="n">
@@ -7050,25 +7045,25 @@
     </row>
     <row r="98" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="s">
+        <v>783</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>772</v>
+      </c>
+      <c r="C98" s="8" t="s">
         <v>784</v>
       </c>
-      <c r="B98" s="8" t="s">
-        <v>773</v>
-      </c>
-      <c r="C98" s="8" t="s">
+      <c r="D98" s="8" t="s">
         <v>785</v>
-      </c>
-      <c r="D98" s="8" t="s">
-        <v>786</v>
       </c>
       <c r="E98" s="8" t="s">
         <v>432</v>
       </c>
       <c r="F98" s="8" t="s">
+        <v>786</v>
+      </c>
+      <c r="G98" s="9" t="s">
         <v>787</v>
-      </c>
-      <c r="G98" s="9" t="s">
-        <v>788</v>
       </c>
       <c r="H98" s="8"/>
       <c r="I98" s="8" t="n">
@@ -7078,25 +7073,25 @@
     </row>
     <row r="99" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="s">
+        <v>788</v>
+      </c>
+      <c r="B99" s="8" t="s">
         <v>789</v>
       </c>
-      <c r="B99" s="8" t="s">
+      <c r="C99" s="8" t="s">
         <v>790</v>
       </c>
-      <c r="C99" s="8" t="s">
+      <c r="D99" s="8" t="s">
         <v>791</v>
-      </c>
-      <c r="D99" s="8" t="s">
-        <v>792</v>
       </c>
       <c r="E99" s="8" t="s">
         <v>281</v>
       </c>
       <c r="F99" s="8" t="s">
+        <v>792</v>
+      </c>
+      <c r="G99" s="9" t="s">
         <v>793</v>
-      </c>
-      <c r="G99" s="9" t="s">
-        <v>794</v>
       </c>
       <c r="H99" s="8"/>
       <c r="I99" s="8" t="n">
@@ -7460,7 +7455,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>205</v>
@@ -7485,7 +7480,7 @@
       <c r="T3" s="13"/>
       <c r="U3" s="13"/>
       <c r="V3" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="W3" s="13"/>
       <c r="X3" s="13"/>
@@ -7500,7 +7495,7 @@
       <c r="AG3" s="13"/>
       <c r="AH3" s="13"/>
       <c r="AI3" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AJ3" s="13"/>
       <c r="AK3" s="13"/>
@@ -7511,7 +7506,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>212</v>
@@ -7541,13 +7536,13 @@
       <c r="Y4" s="13"/>
       <c r="Z4" s="13"/>
       <c r="AA4" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AB4" s="13"/>
       <c r="AC4" s="13"/>
       <c r="AD4" s="13"/>
       <c r="AE4" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AF4" s="13"/>
       <c r="AG4" s="13"/>
@@ -7562,7 +7557,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>218</v>
@@ -7588,11 +7583,11 @@
       <c r="U5" s="13"/>
       <c r="V5" s="13"/>
       <c r="W5" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X5" s="13"/>
       <c r="Y5" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Z5" s="13"/>
       <c r="AA5" s="13"/>
@@ -7613,7 +7608,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>224</v>
@@ -7639,11 +7634,11 @@
       <c r="U6" s="13"/>
       <c r="V6" s="13"/>
       <c r="W6" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X6" s="13"/>
       <c r="Y6" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Z6" s="13"/>
       <c r="AA6" s="13"/>
@@ -7664,7 +7659,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>230</v>
@@ -7692,7 +7687,7 @@
       <c r="W7" s="13"/>
       <c r="X7" s="13"/>
       <c r="Y7" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Z7" s="13"/>
       <c r="AA7" s="13"/>
@@ -7713,7 +7708,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>236</v>
@@ -7731,7 +7726,7 @@
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
       <c r="O8" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="P8" s="13"/>
       <c r="Q8" s="13"/>
@@ -7762,7 +7757,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>243</v>
@@ -7777,7 +7772,7 @@
       <c r="J9" s="13"/>
       <c r="K9" s="13"/>
       <c r="L9" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
@@ -7811,7 +7806,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>249</v>
@@ -7826,7 +7821,7 @@
       <c r="J10" s="13"/>
       <c r="K10" s="13"/>
       <c r="L10" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
@@ -7860,7 +7855,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>255</v>
@@ -7894,7 +7889,7 @@
       <c r="AC11" s="13"/>
       <c r="AD11" s="13"/>
       <c r="AE11" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AF11" s="13"/>
       <c r="AG11" s="13"/>
@@ -7909,7 +7904,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>260</v>
@@ -7943,7 +7938,7 @@
       <c r="AC12" s="13"/>
       <c r="AD12" s="13"/>
       <c r="AE12" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AF12" s="13"/>
       <c r="AG12" s="13"/>
@@ -7958,7 +7953,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>267</v>
@@ -7980,14 +7975,14 @@
       <c r="Q13" s="13"/>
       <c r="R13" s="13"/>
       <c r="S13" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="T13" s="13"/>
       <c r="U13" s="13"/>
       <c r="V13" s="13"/>
       <c r="W13" s="13"/>
       <c r="X13" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Y13" s="13"/>
       <c r="Z13" s="13"/>
@@ -8009,7 +8004,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>274</v>
@@ -8036,10 +8031,10 @@
       <c r="V14" s="13"/>
       <c r="W14" s="13"/>
       <c r="X14" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Y14" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Z14" s="13"/>
       <c r="AA14" s="13"/>
@@ -8060,7 +8055,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>280</v>
@@ -8072,7 +8067,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
       <c r="I15" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="J15" s="13"/>
       <c r="K15" s="13"/>
@@ -8081,7 +8076,7 @@
       <c r="N15" s="13"/>
       <c r="O15" s="13"/>
       <c r="P15" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q15" s="13"/>
       <c r="R15" s="13"/>
@@ -8111,7 +8106,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>287</v>
@@ -8130,7 +8125,7 @@
       <c r="N16" s="13"/>
       <c r="O16" s="13"/>
       <c r="P16" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q16" s="13"/>
       <c r="R16" s="13"/>
@@ -8160,13 +8155,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>293</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D17" s="13"/>
       <c r="E17" s="13"/>
@@ -8183,7 +8178,7 @@
       <c r="P17" s="13"/>
       <c r="Q17" s="13"/>
       <c r="R17" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="S17" s="13"/>
       <c r="T17" s="13"/>
@@ -8211,7 +8206,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>300</v>
@@ -8240,7 +8235,7 @@
       <c r="X18" s="13"/>
       <c r="Y18" s="13"/>
       <c r="Z18" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AA18" s="13"/>
       <c r="AB18" s="13"/>
@@ -8260,7 +8255,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>306</v>
@@ -8285,7 +8280,7 @@
       <c r="T19" s="13"/>
       <c r="U19" s="13"/>
       <c r="V19" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="W19" s="13"/>
       <c r="X19" s="13"/>
@@ -8300,7 +8295,7 @@
       <c r="AG19" s="13"/>
       <c r="AH19" s="13"/>
       <c r="AI19" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AJ19" s="13"/>
       <c r="AK19" s="13"/>
@@ -8311,7 +8306,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>312</v>
@@ -8336,7 +8331,7 @@
       <c r="T20" s="13"/>
       <c r="U20" s="13"/>
       <c r="V20" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="W20" s="13"/>
       <c r="X20" s="13"/>
@@ -8360,7 +8355,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>318</v>
@@ -8375,7 +8370,7 @@
       <c r="J21" s="13"/>
       <c r="K21" s="13"/>
       <c r="L21" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
@@ -8409,7 +8404,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>324</v>
@@ -8442,7 +8437,7 @@
       <c r="AB22" s="13"/>
       <c r="AC22" s="13"/>
       <c r="AD22" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AE22" s="13"/>
       <c r="AF22" s="13"/>
@@ -8458,7 +8453,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>331</v>
@@ -8474,7 +8469,7 @@
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
       <c r="M23" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="N23" s="13"/>
       <c r="O23" s="13"/>
@@ -8507,7 +8502,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>337</v>
@@ -8515,13 +8510,13 @@
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
       <c r="E24" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
       <c r="I24" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="J24" s="13"/>
       <c r="K24" s="13"/>
@@ -8530,7 +8525,7 @@
       <c r="N24" s="13"/>
       <c r="O24" s="13"/>
       <c r="P24" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q24" s="13"/>
       <c r="R24" s="13"/>
@@ -8560,7 +8555,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>343</v>
@@ -8580,7 +8575,7 @@
       <c r="O25" s="13"/>
       <c r="P25" s="13"/>
       <c r="Q25" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="R25" s="13"/>
       <c r="S25" s="13"/>
@@ -8609,7 +8604,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="B26" s="12" t="s">
         <v>348</v>
@@ -8634,7 +8629,7 @@
       <c r="T26" s="13"/>
       <c r="U26" s="13"/>
       <c r="V26" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="W26" s="13"/>
       <c r="X26" s="13"/>
@@ -8649,7 +8644,7 @@
       <c r="AG26" s="13"/>
       <c r="AH26" s="13"/>
       <c r="AI26" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AJ26" s="13"/>
       <c r="AK26" s="13"/>
@@ -8660,7 +8655,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B27" s="12" t="s">
         <v>355</v>
@@ -8684,11 +8679,11 @@
       <c r="S27" s="13"/>
       <c r="T27" s="13"/>
       <c r="U27" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="V27" s="13"/>
       <c r="W27" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X27" s="13"/>
       <c r="Y27" s="13"/>
@@ -8711,7 +8706,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>362</v>
@@ -8744,10 +8739,10 @@
       <c r="AB28" s="13"/>
       <c r="AC28" s="13"/>
       <c r="AD28" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AE28" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AF28" s="13"/>
       <c r="AG28" s="13"/>
@@ -8762,7 +8757,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>368</v>
@@ -8785,10 +8780,10 @@
       <c r="R29" s="13"/>
       <c r="S29" s="13"/>
       <c r="T29" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="U29" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="V29" s="13"/>
       <c r="W29" s="13"/>
@@ -8813,7 +8808,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>374</v>
@@ -8852,7 +8847,7 @@
       <c r="AH30" s="13"/>
       <c r="AI30" s="13"/>
       <c r="AJ30" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AK30" s="13"/>
       <c r="AL30" s="15" t="n">
@@ -8862,16 +8857,16 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>381</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E31" s="13"/>
       <c r="F31" s="13"/>
@@ -8913,7 +8908,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B32" s="12" t="s">
         <v>388</v>
@@ -8922,7 +8917,7 @@
       <c r="D32" s="13"/>
       <c r="E32" s="13"/>
       <c r="F32" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
@@ -8951,7 +8946,7 @@
       <c r="AE32" s="13"/>
       <c r="AF32" s="13"/>
       <c r="AG32" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AH32" s="13"/>
       <c r="AI32" s="13"/>
@@ -8964,7 +8959,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B33" s="12" t="s">
         <v>394</v>
@@ -8990,11 +8985,11 @@
       <c r="U33" s="13"/>
       <c r="V33" s="13"/>
       <c r="W33" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X33" s="13"/>
       <c r="Y33" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Z33" s="13"/>
       <c r="AA33" s="13"/>
@@ -9015,7 +9010,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="B34" s="12" t="s">
         <v>401</v>
@@ -9027,7 +9022,7 @@
       <c r="G34" s="13"/>
       <c r="H34" s="13"/>
       <c r="I34" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="J34" s="13"/>
       <c r="K34" s="13"/>
@@ -9064,7 +9059,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="B35" s="12" t="s">
         <v>407</v>
@@ -9100,7 +9095,7 @@
       <c r="AE35" s="13"/>
       <c r="AF35" s="13"/>
       <c r="AG35" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AH35" s="13"/>
       <c r="AI35" s="13"/>
@@ -9113,7 +9108,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="B36" s="12" t="s">
         <v>413</v>
@@ -9132,7 +9127,7 @@
       <c r="N36" s="13"/>
       <c r="O36" s="13"/>
       <c r="P36" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q36" s="13"/>
       <c r="R36" s="13"/>
@@ -9162,7 +9157,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="B37" s="12" t="s">
         <v>419</v>
@@ -9177,13 +9172,13 @@
       <c r="J37" s="13"/>
       <c r="K37" s="13"/>
       <c r="L37" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="M37" s="13"/>
       <c r="N37" s="13"/>
       <c r="O37" s="13"/>
       <c r="P37" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q37" s="13"/>
       <c r="R37" s="13"/>
@@ -9213,7 +9208,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="B38" s="12" t="s">
         <v>425</v>
@@ -9227,17 +9222,17 @@
       <c r="I38" s="13"/>
       <c r="J38" s="13"/>
       <c r="K38" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="L38" s="13"/>
       <c r="M38" s="13"/>
       <c r="N38" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="O38" s="13"/>
       <c r="P38" s="13"/>
       <c r="Q38" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="R38" s="13"/>
       <c r="S38" s="13"/>
@@ -9266,7 +9261,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="B39" s="12" t="s">
         <v>431</v>
@@ -9274,14 +9269,14 @@
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
       <c r="E39" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="H39" s="13"/>
       <c r="I39" s="13"/>
       <c r="J39" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="K39" s="13"/>
       <c r="L39" s="13"/>
@@ -9317,7 +9312,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="B40" s="12" t="s">
         <v>437</v>
@@ -9333,7 +9328,7 @@
       <c r="K40" s="13"/>
       <c r="L40" s="13"/>
       <c r="M40" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="N40" s="13"/>
       <c r="O40" s="13"/>
@@ -9366,14 +9361,14 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B41" s="12" t="s">
         <v>443</v>
       </c>
       <c r="C41" s="13"/>
       <c r="D41" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E41" s="13"/>
       <c r="F41" s="13"/>
@@ -9405,7 +9400,7 @@
       <c r="AF41" s="13"/>
       <c r="AG41" s="13"/>
       <c r="AH41" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI41" s="13"/>
       <c r="AJ41" s="13"/>
@@ -9417,14 +9412,14 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B42" s="12" t="s">
         <v>448</v>
       </c>
       <c r="C42" s="13"/>
       <c r="D42" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E42" s="13"/>
       <c r="F42" s="13"/>
@@ -9456,7 +9451,7 @@
       <c r="AF42" s="13"/>
       <c r="AG42" s="13"/>
       <c r="AH42" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI42" s="13"/>
       <c r="AJ42" s="13"/>
@@ -9468,7 +9463,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B43" s="12" t="s">
         <v>453</v>
@@ -9497,7 +9492,7 @@
       <c r="X43" s="13"/>
       <c r="Y43" s="13"/>
       <c r="Z43" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AA43" s="13"/>
       <c r="AB43" s="13"/>
@@ -9517,7 +9512,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B44" s="12" t="s">
         <v>459</v>
@@ -9544,11 +9539,11 @@
       <c r="V44" s="13"/>
       <c r="W44" s="13"/>
       <c r="X44" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Y44" s="13"/>
       <c r="Z44" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AA44" s="13"/>
       <c r="AB44" s="13"/>
@@ -9568,7 +9563,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B45" s="12" t="s">
         <v>465</v>
@@ -9589,7 +9584,7 @@
       <c r="P45" s="13"/>
       <c r="Q45" s="13"/>
       <c r="R45" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="S45" s="13"/>
       <c r="T45" s="13"/>
@@ -9599,7 +9594,7 @@
       <c r="X45" s="13"/>
       <c r="Y45" s="13"/>
       <c r="Z45" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AA45" s="13"/>
       <c r="AB45" s="13"/>
@@ -9619,7 +9614,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B46" s="12" t="s">
         <v>471</v>
@@ -9637,10 +9632,10 @@
       <c r="M46" s="13"/>
       <c r="N46" s="13"/>
       <c r="O46" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="P46" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q46" s="13"/>
       <c r="R46" s="13"/>
@@ -9670,7 +9665,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B47" s="12" t="s">
         <v>478</v>
@@ -9695,11 +9690,11 @@
       <c r="T47" s="13"/>
       <c r="U47" s="13"/>
       <c r="V47" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="W47" s="13"/>
       <c r="X47" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Y47" s="13"/>
       <c r="Z47" s="13"/>
@@ -9721,7 +9716,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B48" s="12" t="s">
         <v>484</v>
@@ -9740,7 +9735,7 @@
       <c r="N48" s="13"/>
       <c r="O48" s="13"/>
       <c r="P48" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q48" s="13"/>
       <c r="R48" s="13"/>
@@ -9760,7 +9755,7 @@
       <c r="AF48" s="13"/>
       <c r="AG48" s="13"/>
       <c r="AH48" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI48" s="13"/>
       <c r="AJ48" s="13"/>
@@ -9772,7 +9767,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B49" s="12" t="s">
         <v>491</v>
@@ -9795,7 +9790,7 @@
       <c r="R49" s="13"/>
       <c r="S49" s="13"/>
       <c r="T49" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="U49" s="13"/>
       <c r="V49" s="13"/>
@@ -9821,14 +9816,14 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B50" s="12" t="s">
         <v>497</v>
       </c>
       <c r="C50" s="13"/>
       <c r="D50" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E50" s="13"/>
       <c r="F50" s="13"/>
@@ -9870,7 +9865,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B51" s="12" t="s">
         <v>503</v>
@@ -9897,7 +9892,7 @@
       <c r="V51" s="13"/>
       <c r="W51" s="13"/>
       <c r="X51" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Y51" s="13"/>
       <c r="Z51" s="13"/>
@@ -9919,7 +9914,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B52" s="12" t="s">
         <v>509</v>
@@ -9930,7 +9925,7 @@
       <c r="F52" s="13"/>
       <c r="G52" s="13"/>
       <c r="H52" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="I52" s="13"/>
       <c r="J52" s="13"/>
@@ -9938,12 +9933,12 @@
       <c r="L52" s="13"/>
       <c r="M52" s="13"/>
       <c r="N52" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="O52" s="13"/>
       <c r="P52" s="13"/>
       <c r="Q52" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="R52" s="13"/>
       <c r="S52" s="13"/>
@@ -9972,7 +9967,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B53" s="12" t="s">
         <v>516</v>
@@ -9983,7 +9978,7 @@
       <c r="F53" s="13"/>
       <c r="G53" s="13"/>
       <c r="H53" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="I53" s="13"/>
       <c r="J53" s="13"/>
@@ -10021,7 +10016,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="12" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B54" s="12" t="s">
         <v>521</v>
@@ -10054,7 +10049,7 @@
       <c r="AB54" s="13"/>
       <c r="AC54" s="13"/>
       <c r="AD54" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AE54" s="13"/>
       <c r="AF54" s="13"/>
@@ -10070,7 +10065,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B55" s="12" t="s">
         <v>527</v>
@@ -10101,7 +10096,7 @@
       <c r="Z55" s="13"/>
       <c r="AA55" s="13"/>
       <c r="AB55" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AC55" s="13"/>
       <c r="AD55" s="13"/>
@@ -10119,7 +10114,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B56" s="12" t="s">
         <v>534</v>
@@ -10144,10 +10139,10 @@
       <c r="T56" s="13"/>
       <c r="U56" s="13"/>
       <c r="V56" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="W56" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X56" s="13"/>
       <c r="Y56" s="13"/>
@@ -10161,7 +10156,7 @@
       <c r="AG56" s="13"/>
       <c r="AH56" s="13"/>
       <c r="AI56" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AJ56" s="13"/>
       <c r="AK56" s="13"/>
@@ -10172,7 +10167,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B57" s="12" t="s">
         <v>539</v>
@@ -10212,7 +10207,7 @@
       <c r="AI57" s="13"/>
       <c r="AJ57" s="13"/>
       <c r="AK57" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AL57" s="15" t="n">
         <f aca="false">COUNTIF(C57:AK57,"x")</f>
@@ -10221,7 +10216,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B58" s="12" t="s">
         <v>544</v>
@@ -10233,7 +10228,7 @@
       <c r="G58" s="13"/>
       <c r="H58" s="13"/>
       <c r="I58" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="J58" s="13"/>
       <c r="K58" s="13"/>
@@ -10270,10 +10265,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="C59" s="13"/>
       <c r="D59" s="13"/>
@@ -10290,7 +10285,7 @@
       <c r="O59" s="13"/>
       <c r="P59" s="13"/>
       <c r="Q59" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="R59" s="13"/>
       <c r="S59" s="13"/>
@@ -10303,7 +10298,7 @@
       <c r="Z59" s="13"/>
       <c r="AA59" s="13"/>
       <c r="AB59" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AC59" s="13"/>
       <c r="AD59" s="13"/>
@@ -10321,10 +10316,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="C60" s="13"/>
       <c r="D60" s="13"/>
@@ -10352,10 +10347,10 @@
       <c r="Z60" s="13"/>
       <c r="AA60" s="13"/>
       <c r="AB60" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AC60" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AD60" s="13"/>
       <c r="AE60" s="13"/>
@@ -10372,10 +10367,10 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="C61" s="13"/>
       <c r="D61" s="13"/>
@@ -10407,7 +10402,7 @@
       <c r="AD61" s="13"/>
       <c r="AE61" s="13"/>
       <c r="AF61" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AG61" s="13"/>
       <c r="AH61" s="13"/>
@@ -10421,15 +10416,15 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C62" s="13"/>
       <c r="D62" s="13"/>
       <c r="E62" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="F62" s="13"/>
       <c r="G62" s="13"/>
@@ -10439,7 +10434,7 @@
       <c r="K62" s="13"/>
       <c r="L62" s="13"/>
       <c r="M62" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="N62" s="13"/>
       <c r="O62" s="13"/>
@@ -10472,10 +10467,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C63" s="13"/>
       <c r="D63" s="13"/>
@@ -10497,7 +10492,7 @@
       <c r="T63" s="13"/>
       <c r="U63" s="13"/>
       <c r="V63" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="W63" s="13"/>
       <c r="X63" s="13"/>
@@ -10512,7 +10507,7 @@
       <c r="AG63" s="13"/>
       <c r="AH63" s="13"/>
       <c r="AI63" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AJ63" s="13"/>
       <c r="AK63" s="13"/>
@@ -10523,10 +10518,10 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C64" s="13"/>
       <c r="D64" s="13"/>
@@ -10538,7 +10533,7 @@
       <c r="J64" s="13"/>
       <c r="K64" s="13"/>
       <c r="L64" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="M64" s="13"/>
       <c r="N64" s="13"/>
@@ -10572,10 +10567,10 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="C65" s="13"/>
       <c r="D65" s="13"/>
@@ -10586,10 +10581,10 @@
       <c r="I65" s="13"/>
       <c r="J65" s="13"/>
       <c r="K65" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="L65" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="M65" s="13"/>
       <c r="N65" s="13"/>
@@ -10613,7 +10608,7 @@
       <c r="AF65" s="13"/>
       <c r="AG65" s="13"/>
       <c r="AH65" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI65" s="13"/>
       <c r="AJ65" s="13"/>
@@ -10625,10 +10620,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="12" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C66" s="13"/>
       <c r="D66" s="13"/>
@@ -10659,7 +10654,7 @@
       <c r="AC66" s="13"/>
       <c r="AD66" s="13"/>
       <c r="AE66" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AF66" s="13"/>
       <c r="AG66" s="13"/>
@@ -10674,10 +10669,10 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="12" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B67" s="12" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C67" s="13"/>
       <c r="D67" s="13"/>
@@ -10711,7 +10706,7 @@
       <c r="AF67" s="13"/>
       <c r="AG67" s="13"/>
       <c r="AH67" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI67" s="13"/>
       <c r="AJ67" s="13"/>
@@ -10723,10 +10718,10 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="12" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C68" s="13"/>
       <c r="D68" s="13"/>
@@ -10760,7 +10755,7 @@
       <c r="AF68" s="13"/>
       <c r="AG68" s="13"/>
       <c r="AH68" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI68" s="13"/>
       <c r="AJ68" s="13"/>
@@ -10772,13 +10767,13 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="12" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="13"/>
@@ -10821,10 +10816,10 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="12" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="C70" s="13"/>
       <c r="D70" s="13"/>
@@ -10843,14 +10838,14 @@
       <c r="Q70" s="13"/>
       <c r="R70" s="13"/>
       <c r="S70" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="T70" s="13"/>
       <c r="U70" s="13"/>
       <c r="V70" s="13"/>
       <c r="W70" s="13"/>
       <c r="X70" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Y70" s="13"/>
       <c r="Z70" s="13"/>
@@ -10872,10 +10867,10 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="12" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B71" s="12" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="C71" s="13"/>
       <c r="D71" s="13"/>
@@ -10886,7 +10881,7 @@
       <c r="I71" s="13"/>
       <c r="J71" s="13"/>
       <c r="K71" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="L71" s="13"/>
       <c r="M71" s="13"/>
@@ -10911,7 +10906,7 @@
       <c r="AF71" s="13"/>
       <c r="AG71" s="13"/>
       <c r="AH71" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI71" s="13"/>
       <c r="AJ71" s="13"/>
@@ -10923,10 +10918,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="C72" s="13"/>
       <c r="D72" s="13"/>
@@ -10948,7 +10943,7 @@
       <c r="T72" s="13"/>
       <c r="U72" s="13"/>
       <c r="V72" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="W72" s="13"/>
       <c r="X72" s="13"/>
@@ -10972,10 +10967,10 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C73" s="13"/>
       <c r="D73" s="13"/>
@@ -11003,7 +10998,7 @@
       <c r="Z73" s="13"/>
       <c r="AA73" s="13"/>
       <c r="AB73" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AC73" s="13"/>
       <c r="AD73" s="13"/>
@@ -11021,10 +11016,10 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B74" s="12" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="C74" s="13"/>
       <c r="D74" s="13"/>
@@ -11051,10 +11046,10 @@
       <c r="Y74" s="13"/>
       <c r="Z74" s="13"/>
       <c r="AA74" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AB74" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AC74" s="13"/>
       <c r="AD74" s="13"/>
@@ -11072,10 +11067,10 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="B75" s="12" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="C75" s="13"/>
       <c r="D75" s="13"/>
@@ -11090,7 +11085,7 @@
       <c r="M75" s="13"/>
       <c r="N75" s="13"/>
       <c r="O75" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="P75" s="13"/>
       <c r="Q75" s="13"/>
@@ -11104,10 +11099,10 @@
       <c r="Y75" s="13"/>
       <c r="Z75" s="13"/>
       <c r="AA75" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AB75" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AC75" s="13"/>
       <c r="AD75" s="13"/>
@@ -11125,13 +11120,13 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D76" s="13"/>
       <c r="E76" s="13"/>
@@ -11147,7 +11142,7 @@
       <c r="O76" s="13"/>
       <c r="P76" s="13"/>
       <c r="Q76" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="R76" s="13"/>
       <c r="S76" s="13"/>
@@ -11176,10 +11171,10 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B77" s="12" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="C77" s="13"/>
       <c r="D77" s="13"/>
@@ -11206,7 +11201,7 @@
       <c r="Y77" s="13"/>
       <c r="Z77" s="13"/>
       <c r="AA77" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AB77" s="13"/>
       <c r="AC77" s="13"/>
@@ -11225,10 +11220,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="C78" s="13"/>
       <c r="D78" s="13"/>
@@ -11248,12 +11243,12 @@
       <c r="R78" s="13"/>
       <c r="S78" s="13"/>
       <c r="T78" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="U78" s="13"/>
       <c r="V78" s="13"/>
       <c r="W78" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X78" s="13"/>
       <c r="Y78" s="13"/>
@@ -11276,10 +11271,10 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B79" s="12" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C79" s="13"/>
       <c r="D79" s="13"/>
@@ -11302,11 +11297,11 @@
       <c r="U79" s="13"/>
       <c r="V79" s="13"/>
       <c r="W79" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X79" s="13"/>
       <c r="Y79" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Z79" s="13"/>
       <c r="AA79" s="13"/>
@@ -11318,7 +11313,7 @@
       <c r="AG79" s="13"/>
       <c r="AH79" s="13"/>
       <c r="AI79" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AJ79" s="13"/>
       <c r="AK79" s="13"/>
@@ -11329,10 +11324,10 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B80" s="12" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="C80" s="13"/>
       <c r="D80" s="13"/>
@@ -11354,7 +11349,7 @@
       <c r="T80" s="13"/>
       <c r="U80" s="13"/>
       <c r="V80" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="W80" s="13"/>
       <c r="X80" s="13"/>
@@ -11369,7 +11364,7 @@
       <c r="AG80" s="13"/>
       <c r="AH80" s="13"/>
       <c r="AI80" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AJ80" s="13"/>
       <c r="AK80" s="13"/>
@@ -11380,10 +11375,10 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B81" s="12" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="C81" s="13"/>
       <c r="D81" s="13"/>
@@ -11402,10 +11397,10 @@
       <c r="Q81" s="13"/>
       <c r="R81" s="13"/>
       <c r="S81" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="T81" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="U81" s="13"/>
       <c r="V81" s="13"/>
@@ -11431,13 +11426,13 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="B82" s="12" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D82" s="13"/>
       <c r="E82" s="13"/>
@@ -11457,7 +11452,7 @@
       <c r="S82" s="13"/>
       <c r="T82" s="13"/>
       <c r="U82" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="V82" s="13"/>
       <c r="W82" s="13"/>
@@ -11482,14 +11477,14 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="B83" s="12" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="C83" s="13"/>
       <c r="D83" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E83" s="13"/>
       <c r="F83" s="13"/>
@@ -11521,7 +11516,7 @@
       <c r="AF83" s="13"/>
       <c r="AG83" s="13"/>
       <c r="AH83" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI83" s="13"/>
       <c r="AJ83" s="13"/>
@@ -11533,10 +11528,10 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B84" s="12" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C84" s="13"/>
       <c r="D84" s="13"/>
@@ -11568,7 +11563,7 @@
       <c r="AD84" s="13"/>
       <c r="AE84" s="13"/>
       <c r="AF84" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AG84" s="13"/>
       <c r="AH84" s="13"/>
@@ -11582,10 +11577,10 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B85" s="12" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C85" s="13"/>
       <c r="D85" s="13"/>
@@ -11608,7 +11603,7 @@
       <c r="U85" s="13"/>
       <c r="V85" s="13"/>
       <c r="W85" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X85" s="13"/>
       <c r="Y85" s="13"/>
@@ -11620,7 +11615,7 @@
       <c r="AE85" s="13"/>
       <c r="AF85" s="13"/>
       <c r="AG85" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AH85" s="13"/>
       <c r="AI85" s="13"/>
@@ -11633,10 +11628,10 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B86" s="12" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="C86" s="13"/>
       <c r="D86" s="13"/>
@@ -11659,10 +11654,10 @@
       <c r="U86" s="13"/>
       <c r="V86" s="13"/>
       <c r="W86" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X86" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Y86" s="13"/>
       <c r="Z86" s="13"/>
@@ -11684,10 +11679,10 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B87" s="12" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="C87" s="13"/>
       <c r="D87" s="13"/>
@@ -11702,10 +11697,10 @@
       <c r="M87" s="13"/>
       <c r="N87" s="13"/>
       <c r="O87" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="P87" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="Q87" s="13"/>
       <c r="R87" s="13"/>
@@ -11735,18 +11730,18 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B88" s="12" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="C88" s="13"/>
       <c r="D88" s="13"/>
       <c r="E88" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="F88" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="G88" s="13"/>
       <c r="H88" s="13"/>
@@ -11756,7 +11751,7 @@
       <c r="L88" s="13"/>
       <c r="M88" s="13"/>
       <c r="N88" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="O88" s="13"/>
       <c r="P88" s="13"/>
@@ -11788,10 +11783,10 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B89" s="12" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="C89" s="13"/>
       <c r="D89" s="13"/>
@@ -11821,7 +11816,7 @@
       <c r="AB89" s="13"/>
       <c r="AC89" s="13"/>
       <c r="AD89" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AE89" s="13"/>
       <c r="AF89" s="13"/>
@@ -11837,10 +11832,10 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="12" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B90" s="12" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="C90" s="13"/>
       <c r="D90" s="13"/>
@@ -11850,7 +11845,7 @@
       <c r="H90" s="13"/>
       <c r="I90" s="13"/>
       <c r="J90" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="K90" s="13"/>
       <c r="L90" s="13"/>
@@ -11886,15 +11881,15 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="12" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B91" s="12" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="C91" s="13"/>
       <c r="D91" s="13"/>
       <c r="E91" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="F91" s="13"/>
       <c r="G91" s="13"/>
@@ -11935,14 +11930,14 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="12" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B92" s="12" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="C92" s="13"/>
       <c r="D92" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E92" s="13"/>
       <c r="F92" s="13"/>
@@ -11974,7 +11969,7 @@
       <c r="AF92" s="13"/>
       <c r="AG92" s="13"/>
       <c r="AH92" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI92" s="13"/>
       <c r="AJ92" s="13"/>
@@ -11986,28 +11981,28 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="12" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B93" s="12" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="C93" s="13"/>
       <c r="D93" s="13"/>
       <c r="E93" s="13"/>
       <c r="F93" s="13"/>
       <c r="G93" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="H93" s="13"/>
       <c r="I93" s="13"/>
       <c r="J93" s="13"/>
       <c r="K93" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="L93" s="13"/>
       <c r="M93" s="13"/>
       <c r="N93" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="O93" s="13"/>
       <c r="P93" s="13"/>
@@ -12039,19 +12034,19 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="12" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B94" s="12" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="C94" s="13"/>
       <c r="D94" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E94" s="13"/>
       <c r="F94" s="13"/>
       <c r="G94" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="H94" s="13"/>
       <c r="I94" s="13"/>
@@ -12080,7 +12075,7 @@
       <c r="AF94" s="13"/>
       <c r="AG94" s="13"/>
       <c r="AH94" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="AI94" s="13"/>
       <c r="AJ94" s="13"/>
@@ -12092,10 +12087,10 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="12" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B95" s="12" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="C95" s="13"/>
       <c r="D95" s="13"/>
@@ -12118,7 +12113,7 @@
       <c r="U95" s="13"/>
       <c r="V95" s="13"/>
       <c r="W95" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X95" s="13"/>
       <c r="Y95" s="13"/>
@@ -12141,10 +12136,10 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="12" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B96" s="12" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C96" s="13"/>
       <c r="D96" s="13"/>
@@ -12167,7 +12162,7 @@
       <c r="U96" s="13"/>
       <c r="V96" s="13"/>
       <c r="W96" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="X96" s="13"/>
       <c r="Y96" s="13"/>
@@ -12190,13 +12185,13 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="12" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B97" s="12" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="C97" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D97" s="13"/>
       <c r="E97" s="13"/>
@@ -12204,7 +12199,7 @@
       <c r="G97" s="13"/>
       <c r="H97" s="13"/>
       <c r="I97" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="J97" s="13"/>
       <c r="K97" s="13"/>
@@ -12241,10 +12236,10 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="12" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B98" s="12" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C98" s="13"/>
       <c r="D98" s="13"/>
@@ -12255,7 +12250,7 @@
       <c r="I98" s="13"/>
       <c r="J98" s="13"/>
       <c r="K98" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="L98" s="13"/>
       <c r="M98" s="13"/>
@@ -12290,13 +12285,13 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="12" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B99" s="12" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="C99" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D99" s="13"/>
       <c r="E99" s="13"/>
@@ -12304,7 +12299,7 @@
       <c r="G99" s="13"/>
       <c r="H99" s="13"/>
       <c r="I99" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="J99" s="13"/>
       <c r="K99" s="13"/>
@@ -12341,17 +12336,17 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="12" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="B100" s="12" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="C100" s="13"/>
       <c r="D100" s="13"/>
       <c r="E100" s="13"/>
       <c r="F100" s="13"/>
       <c r="G100" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="H100" s="13"/>
       <c r="I100" s="13"/>
@@ -12360,7 +12355,7 @@
       <c r="L100" s="13"/>
       <c r="M100" s="13"/>
       <c r="N100" s="14" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="O100" s="13"/>
       <c r="P100" s="13"/>

</xml_diff>